<commit_message>
docs: update design source spreadsheet with new content
</commit_message>
<xml_diff>
--- a/docs/product/design-source/蛋仔--大富翁--黑市表.xlsx
+++ b/docs/product/design-source/蛋仔--大富翁--黑市表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lzx_8\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1417645-4073-4C74-B3F2-59C87FEDA277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367783D2-A58A-4006-9153-27478058CC1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -242,23 +242,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,6 +268,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -299,10 +305,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -584,14 +591,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="11.140625" customWidth="1"/>
-    <col min="5" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.125" customWidth="1"/>
+    <col min="5" max="6" width="11.875" customWidth="1"/>
+    <col min="7" max="7" width="10.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -614,7 +621,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -637,7 +644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -650,86 +657,86 @@
       <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="2">
-        <v>2500</v>
-      </c>
-      <c r="G3" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="F3" s="3">
+        <v>5000</v>
+      </c>
+      <c r="G3" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>2005</v>
+        <v>2002</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F4" s="2">
-        <v>2500</v>
-      </c>
-      <c r="G4" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="3">
+        <v>100</v>
+      </c>
+      <c r="G4" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="2">
-        <v>2500</v>
-      </c>
-      <c r="G5" s="2">
+      <c r="E5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="3">
+        <v>200</v>
+      </c>
+      <c r="G5" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <v>2012</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2">
-        <v>2002</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G6" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="G6" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -742,40 +749,40 @@
       <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G7" s="2">
+      <c r="E7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="G7" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>2012</v>
+        <v>2006</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F8" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G8" s="2">
+      <c r="E8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="G8" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -788,17 +795,17 @@
       <c r="D9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="2">
-        <v>100</v>
-      </c>
-      <c r="G9" s="2">
+      <c r="E9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="G9" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -811,17 +818,17 @@
       <c r="D10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="2">
-        <v>100</v>
-      </c>
-      <c r="G10" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="3">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -835,16 +842,16 @@
         <v>7</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F11" s="2">
-        <v>100</v>
-      </c>
-      <c r="G11" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="F11" s="3">
+        <v>10</v>
+      </c>
+      <c r="G11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -860,22 +867,22 @@
       <c r="E12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="2">
-        <v>5</v>
-      </c>
-      <c r="G12" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="F12" s="3">
+        <v>10</v>
+      </c>
+      <c r="G12" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>7</v>
@@ -883,22 +890,22 @@
       <c r="E13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="2">
-        <v>5</v>
-      </c>
-      <c r="G13" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="F13" s="3">
+        <v>10</v>
+      </c>
+      <c r="G13" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>7</v>
@@ -906,22 +913,22 @@
       <c r="E14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="2">
-        <v>5</v>
-      </c>
-      <c r="G14" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="F14" s="3">
+        <v>25</v>
+      </c>
+      <c r="G14" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>7</v>
@@ -929,22 +936,22 @@
       <c r="E15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="2">
-        <v>10</v>
-      </c>
-      <c r="G15" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="F15" s="3">
+        <v>25</v>
+      </c>
+      <c r="G15" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>7</v>
@@ -952,22 +959,22 @@
       <c r="E16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="2">
-        <v>10</v>
-      </c>
-      <c r="G16" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="F16" s="3">
+        <v>25</v>
+      </c>
+      <c r="G16" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>2019</v>
+        <v>2010</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>7</v>
@@ -975,14 +982,14 @@
       <c r="E17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F17" s="2">
-        <v>10</v>
-      </c>
-      <c r="G17" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="F17" s="3">
+        <v>50</v>
+      </c>
+      <c r="G17" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -998,14 +1005,14 @@
       <c r="E18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="2">
-        <v>20</v>
-      </c>
-      <c r="G18" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="F18" s="3">
+        <v>50</v>
+      </c>
+      <c r="G18" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1021,14 +1028,14 @@
       <c r="E19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F19" s="2">
-        <v>20</v>
-      </c>
-      <c r="G19" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="F19" s="3">
+        <v>50</v>
+      </c>
+      <c r="G19" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1044,14 +1051,14 @@
       <c r="E20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F20" s="2">
-        <v>50</v>
-      </c>
-      <c r="G20" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="F20" s="3">
+        <v>100</v>
+      </c>
+      <c r="G20" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1067,14 +1074,14 @@
       <c r="E21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F21" s="2">
-        <v>50</v>
-      </c>
-      <c r="G21" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="F21" s="3">
+        <v>100</v>
+      </c>
+      <c r="G21" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1097,7 +1104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1120,7 +1127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1143,7 +1150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1166,7 +1173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1189,7 +1196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1212,7 +1219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>-1</v>
       </c>
@@ -1235,7 +1242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>-1</v>
       </c>
@@ -1258,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>-1</v>
       </c>
@@ -1281,7 +1288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>-1</v>
       </c>
@@ -1304,7 +1311,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>-1</v>
       </c>
@@ -1327,7 +1334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>-1</v>
       </c>
@@ -1350,7 +1357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>-1</v>
       </c>
@@ -1373,7 +1380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>-1</v>
       </c>
@@ -1396,7 +1403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>-1</v>
       </c>
@@ -1419,7 +1426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>-1</v>
       </c>
@@ -1442,7 +1449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>-1</v>
       </c>
@@ -1465,7 +1472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>-1</v>
       </c>

</xml_diff>